<commit_message>
Update study period to keep context
</commit_message>
<xml_diff>
--- a/characteristics_tables/All_Study_Characteristics.xlsx
+++ b/characteristics_tables/All_Study_Characteristics.xlsx
@@ -499,21 +499,6 @@
           <t>Infants, Children</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
       <c r="I2" t="inlineStr">
         <is>
           <t>16775</t>
@@ -1190,21 +1175,6 @@
       <c r="E9" t="inlineStr">
         <is>
           <t>Adults, Pregnant</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>NR</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -4358,7 +4328,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Pfizer/Moderna COVID - 12/2020 - 01/2022
+          <t>Pfizer/Moderna COVID - 19 vaccine: 12/2020 - 01/2022
 Influenza vaccine: 01/2016 - 01/2022</t>
         </is>
       </c>
@@ -5683,7 +5653,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>04/2021 - 09/2022</t>
+          <t>April 2021 - September 2022</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -7486,7 +7456,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>04/2023 - 04/2024</t>
+          <t>April 2023 - April 2024</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -7786,7 +7756,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>10/2024 - 01/2025</t>
+          <t>October 5, 2024, - January 5, 2025</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -7980,21 +7950,6 @@
           <t>Older Adults</t>
         </is>
       </c>
-      <c r="F75" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="G75" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="H75" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
       <c r="I75" t="inlineStr">
         <is>
           <t>5410</t>
@@ -9070,7 +9025,7 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>05/2022 - 12/2022</t>
+          <t>May 10, 2022 - December 29, 2022</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -9585,7 +9540,7 @@
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>04/2021 - 11/2021 - 12 months post - 2nd vaccine dose</t>
+          <t>04/2021 - 11/2021 (enrollment); followed - 12 months post - 2nd vaccine dose</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
@@ -9992,7 +9947,7 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>03/2021 - 07/2022</t>
+          <t>03/2021 - 07/02/2022</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
@@ -10193,7 +10148,7 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>06/2022 - 06/2023</t>
+          <t>6/01/2022 - 6/01/2023</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
@@ -10497,7 +10452,7 @@
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>03/2022 - 10/2022 - 3 months after 2nd dose or censor</t>
+          <t>03/2022 - 10/2022 (vaccination window); followup - 3 months after 2nd dose or censor</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
@@ -10812,7 +10767,7 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>12/2020 - 04/2022</t>
+          <t>27 December 2020 - 30 April 2022,</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
@@ -10920,7 +10875,7 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>03/2024 - 05/2024 - up 35 days (range 29 - 49 days) at the time of this interim/short - communication analysis</t>
+          <t>03/15/2024 - 05/02/2024 (enrollment); median follow - up 35 days (range 29 - 49 days) at the time of this interim/short - communication analysis</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
@@ -12860,7 +12815,7 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>09/2022 - 02/2024</t>
+          <t>09/ 2022 - 02/2024</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
@@ -14018,7 +13973,7 @@
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>01/2021 - 04/2023
+          <t>Group 1: 01/2021 - 04/2023
 Group 2: 12/2020 - 11/2022
 Group 3: 12/2020 - 10/2022</t>
         </is>
@@ -14432,7 +14387,7 @@
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>04/2024 - 04/2025 (spring campaign), 10/2024 - 04/2025</t>
+          <t>04/2024 - 04/2025 (spring campaign), 10/2024 - 04/2025 (autumn campaign)</t>
         </is>
       </c>
       <c r="G138" t="inlineStr">
@@ -20625,21 +20580,6 @@
           <t>Older Adults, Adults, Pregnant</t>
         </is>
       </c>
-      <c r="F199" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="G199" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="H199" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
       <c r="I199" t="inlineStr">
         <is>
           <t>46913</t>
@@ -21796,7 +21736,7 @@
       </c>
       <c r="F211" t="inlineStr">
         <is>
-          <t>10/2023 - 07/2024</t>
+          <t>24 October 2023 - 26 July 2024</t>
         </is>
       </c>
       <c r="G211" t="inlineStr">
@@ -23502,7 +23442,7 @@
       </c>
       <c r="F228" t="inlineStr">
         <is>
-          <t>09/2021 - 06/2022</t>
+          <t>15 September 2021 - 6 June 2022</t>
         </is>
       </c>
       <c r="G228" t="inlineStr">
@@ -23818,7 +23758,7 @@
       </c>
       <c r="F231" t="inlineStr">
         <is>
-          <t>10/2024 - 05/2025</t>
+          <t>October 1, 2024, - May 31, 2025</t>
         </is>
       </c>
       <c r="G231" t="inlineStr">
@@ -25053,7 +24993,7 @@
       </c>
       <c r="F243" t="inlineStr">
         <is>
-          <t>08/2022 - 03/2024</t>
+          <t>9 August 2022 - 26 March 2024</t>
         </is>
       </c>
       <c r="G243" t="inlineStr">
@@ -27118,7 +27058,7 @@
       </c>
       <c r="F264" t="inlineStr">
         <is>
-          <t>04/2021 - 03/2022</t>
+          <t>13 April 2021 - 3 March 2022</t>
         </is>
       </c>
       <c r="G264" t="inlineStr">
@@ -27314,8 +27254,9 @@
       </c>
       <c r="F266" t="inlineStr">
         <is>
-          <t>05/2023 - 03/2025
-RSVPreF: 5/2023 - 03/2025 - 1345: 5/2024 - 03/2025</t>
+          <t>RSVPreF3: 05/2023 - 03/2025
+RSVPreF: 05/2023 - 03/2025
+mRNA - 1345: 05/2024 - 03/2025</t>
         </is>
       </c>
       <c r="G266" t="inlineStr">
@@ -27708,21 +27649,6 @@
         </is>
       </c>
       <c r="D270" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="F270" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="G270" t="inlineStr">
-        <is>
-          <t>NR</t>
-        </is>
-      </c>
-      <c r="H270" t="inlineStr">
         <is>
           <t>NR</t>
         </is>

</xml_diff>

<commit_message>
Add more clarifying text, remove ecological study design, fix ecological type of outcome filter, add disclaimer
</commit_message>
<xml_diff>
--- a/characteristics_tables/All_Study_Characteristics.xlsx
+++ b/characteristics_tables/All_Study_Characteristics.xlsx
@@ -649,7 +649,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>only 1 arm eligible, treated as single arm</t>
+          <t>primary</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -3633,12 +3633,12 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Non-randomized single arm</t>
+          <t>Observational - with comparator group</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>case series/report</t>
+          <t>SCCS (self-controlled case series)</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
@@ -7587,12 +7587,12 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>Non-randomized single arm</t>
+          <t>Observational - with comparator group</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>case series/report</t>
+          <t>SCCS (self-controlled case series)</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
@@ -7663,12 +7663,12 @@
       </c>
       <c r="Y61" t="inlineStr">
         <is>
-          <t>assessment in progress</t>
+          <t>Critical: D1: Confounding</t>
         </is>
       </c>
       <c r="Z61" t="inlineStr">
         <is>
-          <t>Assessment in Progress</t>
+          <t>Critical</t>
         </is>
       </c>
     </row>
@@ -11220,12 +11220,12 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>Observational - with comparator group</t>
+          <t>Non-randomized single arm</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
         <is>
-          <t>case-control</t>
+          <t>only 1 arm eligible, treated as single arm</t>
         </is>
       </c>
       <c r="L91" t="inlineStr">
@@ -13361,7 +13361,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Mean (SD): Mean (SD): 36.48 ± 0.232</t>
+          <t>NR</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -13386,17 +13386,17 @@
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>2534</t>
+          <t>2031</t>
         </is>
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>Observational - with comparator group</t>
+          <t>Non-randomized single arm</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
         <is>
-          <t>prospective cohort</t>
+          <t>only 1 arm eligible, treated as single arm</t>
         </is>
       </c>
       <c r="L109" t="inlineStr">
@@ -13411,7 +13411,7 @@
       </c>
       <c r="N109" t="inlineStr">
         <is>
-          <t>Other OUS postmarketing registry: Department of Pharmacology at Bangabandhu Sheikh Mujib Medical University (BSMMU)</t>
+          <t>Department of Pharmacology at Bangabandhu Sheikh Mujib Medical University (BSMMU)</t>
         </is>
       </c>
       <c r="O109" t="inlineStr">
@@ -13436,27 +13436,12 @@
       </c>
       <c r="S109" t="inlineStr">
         <is>
-          <t>Grant committee of Bangabandhu Sheikh Mujib Medical University (BSMMU). University research grant Fund. Memo no. 2021-2022/02.</t>
+          <t>This study was supported by the grant committee of Bangabandhu Sheikh Mujib Medical University (BSMMU). University research grant Fund. Memo no. 2021-2022/02</t>
         </is>
       </c>
       <c r="T109" t="inlineStr">
         <is>
           <t>Scientific Reports</t>
-        </is>
-      </c>
-      <c r="U109" t="inlineStr">
-        <is>
-          <t>41006405</t>
-        </is>
-      </c>
-      <c r="V109" t="inlineStr">
-        <is>
-          <t>PMC12475045</t>
-        </is>
-      </c>
-      <c r="W109" t="inlineStr">
-        <is>
-          <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC12475045/</t>
         </is>
       </c>
       <c r="X109" t="inlineStr">
@@ -14001,12 +13986,12 @@
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>Non-randomized single arm</t>
+          <t>Observational - with comparator group</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
         <is>
-          <t>only 1 arm eligible, treated as single arm</t>
+          <t>retrospective cohort</t>
         </is>
       </c>
       <c r="L114" t="inlineStr">
@@ -20546,7 +20531,7 @@
       </c>
       <c r="Q168" t="inlineStr">
         <is>
-          <t>Safety: Other SAEs per study defn, Other SAEs per study defn: Death</t>
+          <t>Safety: Other SAEs per study defn: Death</t>
         </is>
       </c>
       <c r="R168" t="inlineStr">
@@ -26128,12 +26113,12 @@
       </c>
       <c r="J215" t="inlineStr">
         <is>
-          <t>Observational - with comparator group</t>
+          <t>Non-randomized single arm</t>
         </is>
       </c>
       <c r="K215" t="inlineStr">
         <is>
-          <t>retrospective cohort</t>
+          <t>only 1 arm eligible, treated as single arm</t>
         </is>
       </c>
       <c r="L215" t="inlineStr">
@@ -31706,7 +31691,7 @@
       </c>
       <c r="K262" t="inlineStr">
         <is>
-          <t>only 1 arm eligible, treated as single arm</t>
+          <t>primary</t>
         </is>
       </c>
       <c r="L262" t="inlineStr">
@@ -47527,7 +47512,7 @@
         </is>
       </c>
       <c r="D103">
-        <v>2534</v>
+        <v>2031</v>
       </c>
     </row>
     <row r="104">
@@ -81170,7 +81155,12 @@
       </c>
       <c r="D700" t="inlineStr">
         <is>
-          <t>assessment in progress</t>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E700" t="inlineStr">
+        <is>
+          <t>D1: Confounding</t>
         </is>
       </c>
     </row>
@@ -81188,7 +81178,12 @@
       </c>
       <c r="D701" t="inlineStr">
         <is>
-          <t>assessment in progress</t>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E701" t="inlineStr">
+        <is>
+          <t>D1: Confounding</t>
         </is>
       </c>
     </row>
@@ -81206,7 +81201,12 @@
       </c>
       <c r="D702" t="inlineStr">
         <is>
-          <t>assessment in progress</t>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E702" t="inlineStr">
+        <is>
+          <t>D1: Confounding</t>
         </is>
       </c>
     </row>
@@ -81224,7 +81224,12 @@
       </c>
       <c r="D703" t="inlineStr">
         <is>
-          <t>assessment in progress</t>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E703" t="inlineStr">
+        <is>
+          <t>D1: Confounding</t>
         </is>
       </c>
     </row>
@@ -81242,7 +81247,12 @@
       </c>
       <c r="D704" t="inlineStr">
         <is>
-          <t>assessment in progress</t>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E704" t="inlineStr">
+        <is>
+          <t>D1: Confounding</t>
         </is>
       </c>
     </row>
@@ -81260,7 +81270,12 @@
       </c>
       <c r="D705" t="inlineStr">
         <is>
-          <t>assessment in progress</t>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E705" t="inlineStr">
+        <is>
+          <t>D1: Confounding</t>
         </is>
       </c>
     </row>
@@ -81278,7 +81293,12 @@
       </c>
       <c r="D706" t="inlineStr">
         <is>
-          <t>assessment in progress</t>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E706" t="inlineStr">
+        <is>
+          <t>D1: Confounding</t>
         </is>
       </c>
     </row>
@@ -81296,7 +81316,12 @@
       </c>
       <c r="D707" t="inlineStr">
         <is>
-          <t>assessment in progress</t>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E707" t="inlineStr">
+        <is>
+          <t>D1: Confounding</t>
         </is>
       </c>
     </row>
@@ -81314,7 +81339,12 @@
       </c>
       <c r="D708" t="inlineStr">
         <is>
-          <t>assessment in progress</t>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E708" t="inlineStr">
+        <is>
+          <t>D1: Confounding</t>
         </is>
       </c>
     </row>

</xml_diff>